<commit_message>
WBS update 04/24/09:34 tanoue
</commit_message>
<xml_diff>
--- a/Javaシステム開発WBS.xlsx
+++ b/Javaシステム開発WBS.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F83E87F-EB9D-4152-A4AA-8A3523E3FEE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CF35918-B1D1-4DF9-903F-C7242DA0D28D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1849,6 +1849,12 @@
     <xf numFmtId="14" fontId="1" fillId="10" borderId="2" xfId="10" applyNumberFormat="1" applyFill="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="8">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="8" applyBorder="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
     <xf numFmtId="14" fontId="0" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -1860,12 +1866,6 @@
     </xf>
     <xf numFmtId="179" fontId="1" fillId="0" borderId="3" xfId="9">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="8">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="8" applyBorder="1">
-      <alignment horizontal="right" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="54">
@@ -2552,106 +2552,106 @@
       <c r="B3" s="84" t="s">
         <v>142</v>
       </c>
-      <c r="C3" s="101" t="s">
+      <c r="C3" s="97" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="102"/>
-      <c r="E3" s="100">
+      <c r="D3" s="98"/>
+      <c r="E3" s="102">
         <v>45770</v>
       </c>
-      <c r="F3" s="100"/>
+      <c r="F3" s="102"/>
     </row>
     <row r="4" spans="1:64" ht="30" customHeight="1">
       <c r="A4" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="101" t="s">
+      <c r="C4" s="97" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="102"/>
+      <c r="D4" s="98"/>
       <c r="E4" s="4">
         <v>1</v>
       </c>
-      <c r="I4" s="97">
+      <c r="I4" s="99">
         <f>I5</f>
         <v>45768</v>
       </c>
-      <c r="J4" s="98"/>
-      <c r="K4" s="98"/>
-      <c r="L4" s="98"/>
-      <c r="M4" s="98"/>
-      <c r="N4" s="98"/>
-      <c r="O4" s="99"/>
-      <c r="P4" s="97">
+      <c r="J4" s="100"/>
+      <c r="K4" s="100"/>
+      <c r="L4" s="100"/>
+      <c r="M4" s="100"/>
+      <c r="N4" s="100"/>
+      <c r="O4" s="101"/>
+      <c r="P4" s="99">
         <f>P5</f>
         <v>45775</v>
       </c>
-      <c r="Q4" s="98"/>
-      <c r="R4" s="98"/>
-      <c r="S4" s="98"/>
-      <c r="T4" s="98"/>
-      <c r="U4" s="98"/>
-      <c r="V4" s="99"/>
-      <c r="W4" s="97">
+      <c r="Q4" s="100"/>
+      <c r="R4" s="100"/>
+      <c r="S4" s="100"/>
+      <c r="T4" s="100"/>
+      <c r="U4" s="100"/>
+      <c r="V4" s="101"/>
+      <c r="W4" s="99">
         <f>W5</f>
         <v>45782</v>
       </c>
-      <c r="X4" s="98"/>
-      <c r="Y4" s="98"/>
-      <c r="Z4" s="98"/>
-      <c r="AA4" s="98"/>
-      <c r="AB4" s="98"/>
-      <c r="AC4" s="99"/>
-      <c r="AD4" s="97">
+      <c r="X4" s="100"/>
+      <c r="Y4" s="100"/>
+      <c r="Z4" s="100"/>
+      <c r="AA4" s="100"/>
+      <c r="AB4" s="100"/>
+      <c r="AC4" s="101"/>
+      <c r="AD4" s="99">
         <f>AD5</f>
         <v>45789</v>
       </c>
-      <c r="AE4" s="98"/>
-      <c r="AF4" s="98"/>
-      <c r="AG4" s="98"/>
-      <c r="AH4" s="98"/>
-      <c r="AI4" s="98"/>
-      <c r="AJ4" s="99"/>
-      <c r="AK4" s="97">
+      <c r="AE4" s="100"/>
+      <c r="AF4" s="100"/>
+      <c r="AG4" s="100"/>
+      <c r="AH4" s="100"/>
+      <c r="AI4" s="100"/>
+      <c r="AJ4" s="101"/>
+      <c r="AK4" s="99">
         <f>AK5</f>
         <v>45796</v>
       </c>
-      <c r="AL4" s="98"/>
-      <c r="AM4" s="98"/>
-      <c r="AN4" s="98"/>
-      <c r="AO4" s="98"/>
-      <c r="AP4" s="98"/>
-      <c r="AQ4" s="99"/>
-      <c r="AR4" s="97">
+      <c r="AL4" s="100"/>
+      <c r="AM4" s="100"/>
+      <c r="AN4" s="100"/>
+      <c r="AO4" s="100"/>
+      <c r="AP4" s="100"/>
+      <c r="AQ4" s="101"/>
+      <c r="AR4" s="99">
         <f>AR5</f>
         <v>45803</v>
       </c>
-      <c r="AS4" s="98"/>
-      <c r="AT4" s="98"/>
-      <c r="AU4" s="98"/>
-      <c r="AV4" s="98"/>
-      <c r="AW4" s="98"/>
-      <c r="AX4" s="99"/>
-      <c r="AY4" s="97">
+      <c r="AS4" s="100"/>
+      <c r="AT4" s="100"/>
+      <c r="AU4" s="100"/>
+      <c r="AV4" s="100"/>
+      <c r="AW4" s="100"/>
+      <c r="AX4" s="101"/>
+      <c r="AY4" s="99">
         <f>AY5</f>
         <v>45810</v>
       </c>
-      <c r="AZ4" s="98"/>
-      <c r="BA4" s="98"/>
-      <c r="BB4" s="98"/>
-      <c r="BC4" s="98"/>
-      <c r="BD4" s="98"/>
-      <c r="BE4" s="99"/>
-      <c r="BF4" s="97">
+      <c r="AZ4" s="100"/>
+      <c r="BA4" s="100"/>
+      <c r="BB4" s="100"/>
+      <c r="BC4" s="100"/>
+      <c r="BD4" s="100"/>
+      <c r="BE4" s="101"/>
+      <c r="BF4" s="99">
         <f>BF5</f>
         <v>45817</v>
       </c>
-      <c r="BG4" s="98"/>
-      <c r="BH4" s="98"/>
-      <c r="BI4" s="98"/>
-      <c r="BJ4" s="98"/>
-      <c r="BK4" s="98"/>
-      <c r="BL4" s="99"/>
+      <c r="BG4" s="100"/>
+      <c r="BH4" s="100"/>
+      <c r="BI4" s="100"/>
+      <c r="BJ4" s="100"/>
+      <c r="BK4" s="100"/>
+      <c r="BL4" s="101"/>
     </row>
     <row r="5" spans="1:64" ht="15" customHeight="1">
       <c r="A5" s="9" t="s">
@@ -4380,7 +4380,7 @@
         <v>145</v>
       </c>
       <c r="D23" s="42">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E23" s="94">
         <v>45771</v>
@@ -11300,17 +11300,17 @@
     </filterColumn>
   </autoFilter>
   <mergeCells count="11">
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="AK4:AQ4"/>
-    <mergeCell ref="AR4:AX4"/>
-    <mergeCell ref="AY4:BE4"/>
     <mergeCell ref="BF4:BL4"/>
     <mergeCell ref="E3:F3"/>
     <mergeCell ref="I4:O4"/>
     <mergeCell ref="P4:V4"/>
     <mergeCell ref="W4:AC4"/>
     <mergeCell ref="AD4:AJ4"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="AK4:AQ4"/>
+    <mergeCell ref="AR4:AX4"/>
+    <mergeCell ref="AY4:BE4"/>
   </mergeCells>
   <phoneticPr fontId="29"/>
   <conditionalFormatting sqref="D7:D112">
@@ -11487,15 +11487,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="ドキュメント" ma:contentTypeID="0x01010058BEBA3CD4E69545839402B5D4E5400B" ma:contentTypeVersion="13" ma:contentTypeDescription="新しいドキュメントを作成します。" ma:contentTypeScope="" ma:versionID="85fadafb228503a8e253560e9cdffc69">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="88cc3c26-756f-41ab-80ed-43e7289fee5b" xmlns:ns3="55239288-d498-4dd6-9609-491b39ec8fae" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9785dde68d2e35ac7b66dd15e8e44124" ns2:_="" ns3:_="">
     <xsd:import namespace="88cc3c26-756f-41ab-80ed-43e7289fee5b"/>
@@ -11702,6 +11693,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -11714,14 +11714,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4A34E49-7289-4AEA-9593-4F55E04ADB10}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B636D13B-D6CE-437F-B40B-151CC8DA2A1F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11740,6 +11732,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4A34E49-7289-4AEA-9593-4F55E04ADB10}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC3AD2E1-977A-4D4F-8EE8-D64B5FFADF75}">
   <ds:schemaRefs>

</xml_diff>